<commit_message>
Align README statements with v1.0 content
</commit_message>
<xml_diff>
--- a/AI-Risk-Map-Taxonomy-v1.0.xlsx
+++ b/AI-Risk-Map-Taxonomy-v1.0.xlsx
@@ -656,7 +656,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI Risk Map — Working Taxonomy</t>
+          <t>AI Risk Map — Taxonomy Workbook</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr"/>
@@ -757,19 +757,19 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>IMPORTANT: the two-faced splits. Many risks have two legitimate faces owned by different functions. This sheet lists each pair so an apparent duplicate can be checked before it is reported as one.</t>
+          <t>IMPORTANT: the two-faced splits. Many risks have two legitimate faces owned by different functions. This sheet lists each pair with the factor IDs on both faces, so an apparent duplicate can be checked before it is reported as one.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>5. Exclusions register</t>
+          <t>5. Scope decisions</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>What is deliberately OFF the map, and why. Check here before proposing an addition.</t>
+          <t>What is deliberately off the map and why; what was challenged and kept; what was considered and not added. Check here before proposing an addition or reporting a gap.</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Condensed. Full rules, rationale, and rejected alternatives are in AI-Risk-Map-Design-Guide.md, which is the source of truth.</t>
+          <t>Condensed. The full design guide, with rationale and rejected alternatives, is maintained by the author and is not part of this distribution.</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Target 3-4 factors per category, consistent altitude. Do not pad a lean category to hit a quota.</t>
+          <t>Aim for 3–4 factors per category at a consistent altitude; never pad a lean category to hit a quota. v1.0 outcome: mean 3.5 per category, range 2–6, with 48 of 54 categories at 3 or 4.</t>
         </is>
       </c>
     </row>
@@ -1084,440 +1084,440 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Axis</t>
+          <t>Provenance</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Organized by enterprise/management function (who owns the risk), not the AI lifecycle.</t>
+          <t>Each factor tagged to its source framework(s). 'Original' = authored for this map; no reviewed framework names it. See the source-notation legend on this sheet.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>Scope lens</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Risk of ADOPTING AI (others' use of AI against you is out of scope). Within that, incremental-risk only — risks AI introduces or amplifies. Generic IT/cyber risk excluded.</t>
-        </is>
-      </c>
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>HOW TO READ THE SOURCE(S) COLUMN</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Leaf form</t>
+          <t>NAME 0.0</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Each factor is an outcome or condition, never a control or a threat actor.</t>
+          <t>Traces to a specific numbered element in that source (e.g. DASF 5.1, EU Art 14, OWASP LLM01).</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Provenance</t>
+          <t>NAME (no number)</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Each factor tagged to its source framework(s). 'Original' = authored for this map; no reviewed framework names it. See the source-notation legend on this sheet.</t>
+          <t>The concept appears in that source at section or theme level, not as one numbered element.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>HOW TO READ THE SOURCE(S) COLUMN</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr"/>
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Original</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Authored for this map. No reviewed framework names it.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>NAME 0.0</t>
+          <t>NAME; Original</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Traces to a specific numbered element in that source (e.g. DASF 5.1, EU Art 14, OWASP LLM01).</t>
+          <t>The concept traces to that source; the framing and wording are ours. Named sources first, 'Original' always last.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>NAME (no number)</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>The concept appears in that source at section or theme level, not as one numbered element.</t>
+          <t>v1.0 — released. Domains and categories are stable; factors change only through the Change log.</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>Original</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Authored for this map. No reviewed framework names it.</t>
-        </is>
-      </c>
+      <c r="A48" s="3" t="inlineStr"/>
+      <c r="B48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>NAME; Original</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>The concept traces to that source; the framing and wording are ours. Named sources first, 'Original' always last.</t>
-        </is>
-      </c>
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>License and attribution</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>License</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>L1 &amp; L2 LOCKED. Tier 3 populated and validated. v1.0.</t>
+          <t>AI Risk Map (c) 2026 Evan Wheeler. Licensed under Creative Commons Attribution-ShareAlike 4.0 International (CC BY-SA 4.0).</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr"/>
-      <c r="B51" s="2" t="inlineStr"/>
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>License terms</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>https://creativecommons.org/licenses/by-sa/4.0/</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>License and attribution</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr"/>
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>You may</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Share and adapt this work, including commercially.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>License</t>
+          <t>You must</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>AI Risk Map (c) 2026 Evan Wheeler. Licensed under Creative Commons Attribution-ShareAlike 4.0 International (CC BY-SA 4.0).</t>
+          <t>(1) Give appropriate credit: "AI Risk Map (c) 2026 Evan Wheeler, CC BY-SA 4.0"; (2) indicate if changes were made; (3) license any adaptation under CC BY-SA 4.0.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>License terms</t>
+          <t>Source attribution</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>https://creativecommons.org/licenses/by-sa/4.0/</t>
+          <t>Databricks AI Security Framework (DASF) v3.0 and Databricks AI Governance Framework v1.0 are (c) Databricks, licensed CC BY-SA 4.0; this work adapts material from both. The MIT AI Risk Repository is (c) MIT FutureTech, licensed CC BY 4.0; its sub-domain numbering is used in citations.</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="3" t="inlineStr">
-        <is>
-          <t>You may</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>Share and adapt this work, including commercially.</t>
-        </is>
-      </c>
+      <c r="A55" s="3" t="inlineStr"/>
+      <c r="B55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="inlineStr">
-        <is>
-          <t>You must</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>(1) Give appropriate credit: "AI Risk Map (c) 2026 Evan Wheeler, CC BY-SA 4.0"; (2) indicate if changes were made; (3) license any adaptation under CC BY-SA 4.0.</t>
-        </is>
-      </c>
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Poster footnotes (rendered verbatim on the poster)</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Source attribution</t>
+          <t>1. Form</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Databricks AI Security Framework (DASF) v3.0 and Databricks AI Governance Framework v1.0 are (c) Databricks, licensed CC BY-SA 4.0. This work adapts material from both.</t>
+          <t>each entry is a risk FACTOR: a condition, failure mode, or event that contributes to risk. Scope it before analysis.</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr"/>
-      <c r="B58" s="2" t="inlineStr"/>
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>2. Quantification</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>some factors scope cleanly into CRQ/FAIR scenarios; others are board-narrative.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>Methodology caveats (poster footnotes)</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr"/>
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>3. Likelihood</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>position and size do not imply likelihood or severity; rare high-impact factors sit beside common ones.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>1. Scope</t>
+          <t>4. Use</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>These are risk categories to identify and scope — each leaf is a prompt for analysis, not a quantified or measured risk.</t>
+          <t>this map seeds threat modeling and risk assessment; it complements, it does not replace, system-specific models.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>2. Quantification</t>
+          <t>5. Scope</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Some leaves are quantifiable (scopeable into CRQ/FAIR scenarios); others are board-narrative. Treat each accordingly.</t>
+          <t>risks from your organization's adoption of AI; others' use of AI against you belongs on your threat register. Not exhaustive; customize to your context.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>3. Likelihood</t>
+          <t>»n</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Position and size on the map do not imply likelihood or severity — a rare, high-impact risk may sit beside a common one.</t>
+          <t>»n = a related factor owned by domain n, the same risk from that function's angle. Color matches the domain; full descriptions in the workbook.</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="3" t="inlineStr">
-        <is>
-          <t>4. Use</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>This map seeds threat modeling and risk assessment; it complements, it does not replace, system-specific threat models.</t>
-        </is>
-      </c>
+      <c r="A63" s="3" t="inlineStr"/>
+      <c r="B63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="inlineStr">
-        <is>
-          <t>5. Not exhaustive</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>A guide to broaden perspective, not a definitive list. Customize to your industry, geography, and context.</t>
-        </is>
-      </c>
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>Source key</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="inlineStr"/>
-      <c r="B65" s="2" t="inlineStr"/>
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>NIST GenAI #n</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>NIST AI 600-1 GenAI Profile — 12 risk categories</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" s="4" t="inlineStr">
-        <is>
-          <t>Source key</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr"/>
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>NIST Govern/Map/Measure/Manage</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>NIST AI RMF 1.0 — core functions</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>NIST GenAI #n</t>
+          <t>EU Art n</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>NIST AI 600-1 GenAI Profile — 12 risk categories</t>
+          <t>EU AI Act (Reg. 2024/1689, as amended 2026) — articles; '(amended 2026)' = changed by the Digital Omnibus</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>NIST Govern/Map/Measure/Manage</t>
+          <t>GDPR</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>NIST AI RMF 1.0 — core functions</t>
+          <t>GDPR — document level</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>EU Art n</t>
+          <t>ISO A.n</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>EU AI Act (Reg. 2024/1689, as amended 2026) — articles; '(amended 2026)' = changed by the Digital Omnibus</t>
+          <t>ISO/IEC 42001 — Annex A control objectives</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>GDPR</t>
+          <t>OWASP LLMnn</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>GDPR — document level</t>
+          <t>OWASP Top 10 for LLM Applications 2025</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>ISO A.n</t>
+          <t>OWASP ASI Tn</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>ISO/IEC 42001 — Annex A control objectives</t>
+          <t>OWASP Agentic AI — Threats &amp; Mitigations — threat IDs T1–T15 from the OWASP Agentic Security Initiative guide; the separate Top 10 for Agentic Applications numbers ASI01–ASI10</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>OWASP LLMnn</t>
+          <t>OWASP AISVS n.n.n / AC.n</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>OWASP Top 10 for LLM Applications 2025</t>
+          <t>OWASP AISVS 1.0 — requirements; AC = Appendix C</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>OWASP ASI Tn</t>
+          <t>OWASP</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>OWASP Top 10 for Agentic Applications — threat IDs</t>
+          <t>OWASP (other)</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>OWASP AISVS n.n.n / AC.n</t>
+          <t>ATLAS AML.Tnnnn</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>OWASP AISVS 1.0 — requirements; AC = Appendix C</t>
+          <t>MITRE ATLAS — technique IDs</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>OWASP</t>
+          <t>DASF n.n</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>OWASP (other)</t>
+          <t>Databricks AI Security Framework v3.0 — risk IDs</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>ATLAS AML.Tnnnn</t>
+          <t>Databricks AIGF</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>MITRE ATLAS — technique IDs</t>
+          <t>Databricks AI Governance Framework — 5 pillars</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>DASF n.n</t>
+          <t>COSO GenAI 2026</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Databricks AI Security Framework v3.0 — risk IDs</t>
+          <t>COSO — Internal Control over GenAI (2026) — principles</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Databricks AIGF</t>
+          <t>CRI XX-n.n.n</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Databricks AI Governance Framework — 5 pillars</t>
+          <t>CRI Financial Services AI RMF v1.0 — control-objective IDs</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>COSO GenAI 2026</t>
+          <t>CoSAI AI SRF</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>COSO — Internal Control over GenAI (2026) — principles</t>
+          <t>CoSAI AI Shared Responsibility Framework — five-layer accountability model</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>CRI XX-n.n.n</t>
+          <t>Cisco/VAIL provenance-entanglement research 2026</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>CRI Financial Services AI RMF v1.0 — control-objective IDs</t>
+          <t>Cisco / VAIL 'Models Don't Have Passports' (2026) — model-lineage fingerprinting study</t>
         </is>
       </c>
     </row>
@@ -9052,7 +9052,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Excluded by form; leaves are risk statements, not 'MFA' or 'an attacker'.</t>
+          <t>Excluded by form; entries are risk factors — conditions and failure modes — never a control ('MFA') or a threat actor ('an attacker').</t>
         </is>
       </c>
     </row>
@@ -9687,7 +9687,7 @@
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>First public release. 12 domains, 54 categories, 189 risk factors, each with a permanent identifier (AIRM-001 onward). Structure: organized by the enterprise function that owns the risk, not by AI lifecycle. Scope: risk arising from the organization's own adoption of AI. Validation before release: crosswalked against fifteen frameworks and regulations; persona and named-expert critique; five rounds of external practitioner review; used as the validation standard for an independent 264-control catalog; and a full citation audit in which every named source locator was verified against the primary text and every factor tagged Original was checked against every cited framework. Result: 189 of 189 factors traceable; 98 carry the author's framing; 30 are named by no reviewed framework. From this version, changes are recorded at factor grain on the Change log sheet, and identifiers never change.</t>
+          <t>First public release. 12 domains, 54 categories, 189 risk factors, each with a permanent identifier (AIRM-001 onward). Structure: organized by the enterprise function that owns the risk, not by AI lifecycle. Scope: risk arising from the organization's own adoption of AI. Validation before release: crosswalked against 22 frameworks, regulations, and taxonomies; persona and named-expert critique; several rounds of external practitioner review; used as the validation standard for an independent 264-control catalog; and a full citation audit in which every named source locator was verified against the primary text and every factor tagged Original was checked against every cited framework. Result: 189 of 189 factors traceable; 98 carry the author's framing; 30 are named by no reviewed framework. From this version, changes are recorded at factor grain on the Change log sheet, and identifiers never change.</t>
         </is>
       </c>
     </row>

</xml_diff>